<commit_message>
Correction to AHI sensor
</commit_message>
<xml_diff>
--- a/data/cci/cci-sensor.xlsx
+++ b/data/cci/cci-sensor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stfc365-my.sharepoint.com/personal/alison_waterfall_stfc_ac_uk/Documents/Documents/GitHub/cci-vocabularies/data/cci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{26BBE7DF-4C63-4A86-92DF-2DFFF951F08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C59D353-B00D-479B-B3EA-622C9CE63562}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{26BBE7DF-4C63-4A86-92DF-2DFFF951F08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9C32BE0-CB86-4E08-B1F4-9E11164180FD}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="34515" windowHeight="15285" xr2:uid="{AC6267AA-9592-A246-9899-93CEA800D98F}"/>
+    <workbookView xWindow="39105" yWindow="2940" windowWidth="34515" windowHeight="15285" xr2:uid="{AC6267AA-9592-A246-9899-93CEA800D98F}"/>
   </bookViews>
   <sheets>
     <sheet name="cci-sensor" sheetId="1" r:id="rId1"/>
@@ -1266,9 +1266,6 @@
     <t>https://space.oscar.wmo.int/instruments/view/mopitt</t>
   </si>
   <si>
-    <t>sen_ahi</t>
-  </si>
-  <si>
     <t>AHI</t>
   </si>
   <si>
@@ -1276,6 +1273,9 @@
   </si>
   <si>
     <t>https://space.oscar.wmo.int/instruments/view/ahi</t>
+  </si>
+  <si>
+    <t>sens_ahi</t>
   </si>
 </sst>
 </file>
@@ -4459,16 +4459,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
+        <v>417</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="D103" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="D103" s="3" t="s">
+      <c r="E103" s="9" t="s">
         <v>416</v>
-      </c>
-      <c r="E103" s="9" t="s">
-        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>